<commit_message>
Calculo schedule teniendo en cuenta TIMEZONE. Permissions para todos los jobs (ya no por job).
</commit_message>
<xml_diff>
--- a/automatize_predict/update_predictions/schedules.xlsx
+++ b/automatize_predict/update_predictions/schedules.xlsx
@@ -457,7 +457,7 @@
         <v>167</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45462.96875</v>
+        <v>45463.09375</v>
       </c>
     </row>
     <row r="3">
@@ -468,7 +468,7 @@
         <v>167</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45462.97916666666</v>
+        <v>45463.10416666666</v>
       </c>
     </row>
     <row r="4">
@@ -479,7 +479,7 @@
         <v>167</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>45463.01041666666</v>
+        <v>45463.13541666666</v>
       </c>
     </row>
     <row r="5">
@@ -490,7 +490,7 @@
         <v>167</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>45463.09375</v>
+        <v>45463.21875</v>
       </c>
     </row>
     <row r="6">
@@ -501,7 +501,7 @@
         <v>167</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>45465.96875</v>
+        <v>45466.09375</v>
       </c>
     </row>
     <row r="7">
@@ -512,7 +512,7 @@
         <v>167</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>45466.01041666666</v>
+        <v>45466.13541666666</v>
       </c>
     </row>
     <row r="8">
@@ -523,7 +523,7 @@
         <v>167</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>45466.05208333334</v>
+        <v>45466.17708333334</v>
       </c>
     </row>
     <row r="9">
@@ -534,7 +534,7 @@
         <v>167</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>45466.09375</v>
+        <v>45466.21875</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Schedules a partir de df_historial_predicciones
</commit_message>
<xml_diff>
--- a/automatize_predict/update_predictions/schedules.xlsx
+++ b/automatize_predict/update_predictions/schedules.xlsx
@@ -451,90 +451,90 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>45462.97916666666</v>
+        <v>45462.85416666666</v>
       </c>
       <c r="B2" t="n">
         <v>167</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45463.09375</v>
+        <v>45462.96875</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45462.98958333334</v>
+        <v>45462.86458333334</v>
       </c>
       <c r="B3" t="n">
         <v>167</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45463.10416666666</v>
+        <v>45462.97916666666</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45463.02083333334</v>
+        <v>45462.89583333334</v>
       </c>
       <c r="B4" t="n">
         <v>167</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>45463.13541666666</v>
+        <v>45463.01041666666</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45463.10416666666</v>
+        <v>45462.97916666666</v>
       </c>
       <c r="B5" t="n">
         <v>167</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>45463.21875</v>
+        <v>45463.09375</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45465.97916666666</v>
+        <v>45465.85416666666</v>
       </c>
       <c r="B6" t="n">
         <v>167</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>45466.09375</v>
+        <v>45465.96875</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45466.02083333334</v>
+        <v>45465.89583333334</v>
       </c>
       <c r="B7" t="n">
         <v>167</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>45466.13541666666</v>
+        <v>45466.01041666666</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45466.0625</v>
+        <v>45465.9375</v>
       </c>
       <c r="B8" t="n">
         <v>167</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>45466.17708333334</v>
+        <v>45466.05208333334</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45466.10416666666</v>
+        <v>45465.97916666666</v>
       </c>
       <c r="B9" t="n">
         <v>167</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>45466.21875</v>
+        <v>45466.09375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizo push y argumentos de collect_predictions.py
</commit_message>
<xml_diff>
--- a/automatize_predict/update_predictions/schedules.xlsx
+++ b/automatize_predict/update_predictions/schedules.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,90 +451,46 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>45462.85416666666</v>
+        <v>45462.97916666666</v>
       </c>
       <c r="B2" t="n">
         <v>167</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45462.96875</v>
+        <v>45463.09375</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45462.86458333334</v>
+        <v>45462.98958333334</v>
       </c>
       <c r="B3" t="n">
         <v>167</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45462.97916666666</v>
+        <v>45463.10416666666</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45462.89583333334</v>
+        <v>45463.02083333334</v>
       </c>
       <c r="B4" t="n">
         <v>167</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>45463.01041666666</v>
+        <v>45463.13541666666</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45462.97916666666</v>
+        <v>45463.10416666666</v>
       </c>
       <c r="B5" t="n">
         <v>167</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>45463.09375</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>45465.85416666666</v>
-      </c>
-      <c r="B6" t="n">
-        <v>167</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>45465.96875</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>45465.89583333334</v>
-      </c>
-      <c r="B7" t="n">
-        <v>167</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>45466.01041666666</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>45465.9375</v>
-      </c>
-      <c r="B8" t="n">
-        <v>167</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>45466.05208333334</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>45465.97916666666</v>
-      </c>
-      <c r="B9" t="n">
-        <v>167</v>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>45466.09375</v>
+        <v>45463.21875</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fallo el horario en que se corrieron los update
</commit_message>
<xml_diff>
--- a/automatize_predict/update_predictions/schedules.xlsx
+++ b/automatize_predict/update_predictions/schedules.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,45 +451,23 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>45462.97916666666</v>
+        <v>45463.02083333334</v>
       </c>
       <c r="B2" t="n">
         <v>167</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45463.09375</v>
+        <v>45463.13541666666</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45462.98958333334</v>
+        <v>45463.10416666666</v>
       </c>
       <c r="B3" t="n">
         <v>167</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45463.10416666666</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>45463.02083333334</v>
-      </c>
-      <c r="B4" t="n">
-        <v>167</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>45463.13541666666</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>45463.10416666666</v>
-      </c>
-      <c r="B5" t="n">
-        <v>167</v>
-      </c>
-      <c r="C5" s="2" t="n">
         <v>45463.21875</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Arreglo horario de schedules.xslx
</commit_message>
<xml_diff>
--- a/automatize_predict/update_predictions/schedules.xlsx
+++ b/automatize_predict/update_predictions/schedules.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,24 +451,46 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>45463.02083333334</v>
+        <v>45462.97916666666</v>
       </c>
       <c r="B2" t="n">
         <v>167</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45463.13541666666</v>
+        <v>45462.96875</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45463.10416666666</v>
+        <v>45462.98958333334</v>
       </c>
       <c r="B3" t="n">
         <v>167</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45463.21875</v>
+        <v>45462.97916666666</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>45463.02083333334</v>
+      </c>
+      <c r="B4" t="n">
+        <v>167</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>45463.01041666666</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>45463.10416666666</v>
+      </c>
+      <c r="B5" t="n">
+        <v>167</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>45463.09375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ineficiencia en extraction de datos y arreglo de errores en automatización de predict - Extraccion de next_matches. Evito extraer stats (no se por que no lo evitaba… si los próximos partidos no tienen stats puesto que no se jugaron aun)
- Automatización de main_next_matches
    - collect_predictions.py: Simplifico el agregado de predicciones.xlsx a historial_predicciones.xlsx (y lo arreglo pues el historial se borraba…)
    - create_action_update: Quito el delta de hora por la diferencia de Argentina de 3 horas respecto de UTC. Esto es porque cuando extraigo partidos desde la máquina de Gihub, se extrae en horario UTC.
</commit_message>
<xml_diff>
--- a/automatize_predict/update_predictions/schedules.xlsx
+++ b/automatize_predict/update_predictions/schedules.xlsx
@@ -451,46 +451,46 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>45462.97916666666</v>
+        <v>45465.85416666666</v>
       </c>
       <c r="B2" t="n">
         <v>167</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45463.09375</v>
+        <v>45465.96875</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45462.98958333334</v>
+        <v>45465.89583333334</v>
       </c>
       <c r="B3" t="n">
         <v>167</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45463.10416666666</v>
+        <v>45466.01041666666</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45463.02083333334</v>
+        <v>45465.9375</v>
       </c>
       <c r="B4" t="n">
         <v>167</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>45463.13541666666</v>
+        <v>45466.05208333334</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45463.10416666666</v>
+        <v>45465.97916666666</v>
       </c>
       <c r="B5" t="n">
         <v>167</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>45463.21875</v>
+        <v>45466.09375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Get predictions next 15 days
</commit_message>
<xml_diff>
--- a/automatize_predict/update_predictions/schedules.xlsx
+++ b/automatize_predict/update_predictions/schedules.xlsx
@@ -451,7 +451,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>45465.85416666666</v>
+        <v>45465.97916666666</v>
       </c>
       <c r="B2" t="n">
         <v>167</v>
@@ -462,7 +462,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45465.89583333334</v>
+        <v>45466.02083333334</v>
       </c>
       <c r="B3" t="n">
         <v>167</v>
@@ -473,7 +473,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45465.9375</v>
+        <v>45466.0625</v>
       </c>
       <c r="B4" t="n">
         <v>167</v>
@@ -484,7 +484,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45465.97916666666</v>
+        <v>45466.10416666666</v>
       </c>
       <c r="B5" t="n">
         <v>167</v>

</xml_diff>